<commit_message>
Add priced floor-by-floor BOQ in client format; align verified BOQ
Priced BOQ (GHS) built on the client template: substructure, ground to
12th level bills, lifts & provisional sums, priced preliminaries, and a
RATES sheet that every rate links to. Verified BOQ updated for 23 stair
storey-flights and per-floor blockwork/hinge totals.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017tF8o5Ym6pexSoVPAxHdLA
</commit_message>
<xml_diff>
--- a/KANESHIE_BLOCK_N_BOQ_rev1_VERIFIED.xlsx
+++ b/KANESHIE_BLOCK_N_BOQ_rev1_VERIFIED.xlsx
@@ -7985,7 +7985,7 @@
       </c>
       <c r="D102" s="192">
         <f>'Verification Take-off'!E35</f>
-        <v>124.5299393939394</v>
+        <v>127.1549393939394</v>
       </c>
       <c r="E102" s="56" t="inlineStr">
         <is>
@@ -9153,7 +9153,7 @@
       <c r="C150" s="198" t="n"/>
       <c r="D150" s="192">
         <f>'Verification Take-off'!E62</f>
-        <v>731.8607999999999</v>
+        <v>765.1271999999999</v>
       </c>
       <c r="E150" s="196" t="inlineStr">
         <is>
@@ -13771,7 +13771,7 @@
       </c>
       <c r="D12" s="162">
         <f>'Verification Take-off'!E67</f>
-        <v>14110.532118399999</v>
+        <v>14146.501749599995</v>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
@@ -14005,7 +14005,7 @@
       <c r="C13" s="180" t="n"/>
       <c r="D13" s="162">
         <f>'Verification Take-off'!E68</f>
-        <v>1744.1390815999998</v>
+        <v>1708.1694503999997</v>
       </c>
       <c r="E13" s="178" t="inlineStr">
         <is>
@@ -16348,7 +16348,7 @@
       </c>
       <c r="D62" s="162">
         <f>'Verification Take-off'!E86</f>
-        <v>8342.48</v>
+        <v>8374.22</v>
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
@@ -16488,7 +16488,7 @@
       </c>
       <c r="D70" s="223">
         <f>'Verification Take-off'!E78</f>
-        <v>698.2800000000001</v>
+        <v>730.0200000000001</v>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
@@ -18428,7 +18428,7 @@
       </c>
       <c r="D151" s="162">
         <f>'Verification Take-off'!E101</f>
-        <v>449.0</v>
+        <v>452.0</v>
       </c>
       <c r="E151" s="11" t="inlineStr">
         <is>
@@ -30202,17 +30202,17 @@
       </c>
       <c r="C35" s="254" t="inlineStr">
         <is>
-          <t>Stairs: per storey 2 flights (waist 175, 1800 wide, 3.0m going) + 2 landings; scaled to storey height. Main 10 storeys (sum H 37.0m), emergency 12 storeys (sum H 37.3m)</t>
+          <t>Stairs: per storey 2 flights (waist 175, 1800 wide, 3.0m going) + 2 landings; scaled to storey height. Main 11 storeys (sum H 37.0m), emergency 12 storeys (sum H 37.3m)</t>
         </is>
       </c>
       <c r="D35" s="254" t="inlineStr">
         <is>
-          <t>'=2.966*(37.0+37.3)/3.3+2.625*(10+12)</t>
+          <t>'=2.966*(37.0+37.3)/3.3+2.625*(11+12)</t>
         </is>
       </c>
       <c r="E35" s="255">
-        <f>2.966*(37.0+37.3)/3.3+2.625*(10+12)</f>
-        <v>124.5299393939394</v>
+        <f>2.966*(37.0+37.3)/3.3+2.625*(11+12)</f>
+        <v>127.1549393939394</v>
       </c>
       <c r="F35" s="254" t="inlineStr">
         <is>
@@ -31068,17 +31068,17 @@
       </c>
       <c r="C62" s="254" t="inlineStr">
         <is>
-          <t>Stair soffits &amp; risers (per storey 33.3 m2 x 22 storey-flights)</t>
+          <t>Stair soffits &amp; risers (per storey 33.3 m2 x 23 storey-flights)</t>
         </is>
       </c>
       <c r="D62" s="254" t="inlineStr">
         <is>
-          <t>'=(2*3.424*1.8+15.0+22*0.15*1.8)*22</t>
+          <t>'=(2*3.424*1.8+15.0+22*0.15*1.8)*23</t>
         </is>
       </c>
       <c r="E62" s="255">
-        <f>(2*3.424*1.8+15.0+22*0.15*1.8)*22</f>
-        <v>731.8607999999999</v>
+        <f>(2*3.424*1.8+15.0+22*0.15*1.8)*23</f>
+        <v>765.1271999999999</v>
       </c>
       <c r="F62" s="254" t="inlineStr">
         <is>
@@ -31219,17 +31219,17 @@
       </c>
       <c r="C67" s="254" t="inlineStr">
         <is>
-          <t>150mm sandcrete blockwork</t>
+          <t>150mm sandcrete blockwork (sum of floor-by-floor measurement incl. add-back over openings per floor)</t>
         </is>
       </c>
       <c r="D67" s="254" t="inlineStr">
         <is>
-          <t>'=E64+E66*0.882</t>
+          <t>'=203.6*3.6+(1*1.8*(3.05-2.4)+6*0.9*(3.05-2.2)+1*0.9*(3.05-2.35)+1*3.2*(3.05-2.2)+6*0.75*(3.05-2.2)+2*0.7*(3.05-2.2)+3*1*(3.05-2.2)+2*0.9*(3.05-2.2)+3*1.8*(3.05-2.2)+2*1.8*(3.05-2.2)+2*2.4*(3.05-2.2)+1*5.05*(3.05-2.2)+2*4.2*(3.05-2.157)+1*3.6*(3.05-1.9)+1*1.8*(3.05-1.5)+1*1.8*(3.05-1.9)+1*3.5*(3.05-1.5)+3*3.6*(3.05-2.2)+2*2.4*(3.05-1.9)+2*2.1*(3.05-0.9)+4*0.9*(3.05-0.6)+1*0.75*(3.05-0.6))*0.858+98.4*2.45+(3*1*(3.05-2.2))*0.729+144.5*2.45+(3*1*(3.05-2.2))*0.896+127.5*2.45+(3*1*(3.05-2.2))*0.801+500.0*3.05+(10*1*(3.05-2.2)+19*0.9*(3.05-2.2)+21*0.75*(3.05-2.2)+2*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+2*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+3*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+3*1.3*(3.05-2.2)+5*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+7*1.8*(3.05-1.3)+13*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+4*1.2*(3.05-1.9)+10*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+8*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+4*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+12*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.914+443.9*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+22*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+2*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+3*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+7*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+13*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+2*0.6*(3.05-0.6)+2*1.2*(3.05-0.6))*0.889+447.7*3.05+(7*1*(3.05-2.2)+15*0.9*(3.05-2.2)+20*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+3*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+3*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+12*0.9*(3.05-0.6)+4*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.901+465.9*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+21*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+13*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+2*0.6*(3.05-0.6)+2*1.2*(3.05-0.6))*0.903+449.8*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+20*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+3*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+12*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.900+441.2*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+21*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1.2*(3.05-2.2)+3*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+13*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+2*0.6*(3.05-0.6)+2*1.2*(3.05-0.6))*0.895+397.2*3.05+(4*1*(3.05-2.2)+8*0.9*(3.05-2.2)+17*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1.2*(3.05-2.2)+2*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+2*1.6*(3.05-2.2)+1*1.3*(3.05-2.2)+2*1.8*(3.05-2.2)+3*1.8*(3.05-1.3)+6*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+1*1.2*(3.05-1.9)+5*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+3*1.5*(3.05-1.3)+2*1.5*(3.05-1.15)+1*3*(3.05-1.6)+1*1.8*(3.05-1.9)+10*0.9*(3.05-0.6)+4*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.940+354.0*3.05+(6*1*(3.05-2.2)+11*0.9*(3.05-2.2)+16*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1.2*(3.05-2.2)+2*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+3*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+3*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+4*1.8*(3.05-1.3)+8*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+2*1.2*(3.05-1.9)+6*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+5*1.5*(3.05-1.3)+3*1.5*(3.05-1.15)+1*3*(3.05-1.6)+2*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+10*0.9*(3.05-0.6)+4*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.919+82.0*2.9+(7*0.9*(3.05-2.2)+8*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+5*0.9*(3.05-0.6)+2*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.890+6.5*1.2</t>
         </is>
       </c>
       <c r="E67" s="255">
-        <f>E64+E66*0.882</f>
-        <v>14110.532118399999</v>
+        <f>203.6*3.6+(1*1.8*(3.05-2.4)+6*0.9*(3.05-2.2)+1*0.9*(3.05-2.35)+1*3.2*(3.05-2.2)+6*0.75*(3.05-2.2)+2*0.7*(3.05-2.2)+3*1*(3.05-2.2)+2*0.9*(3.05-2.2)+3*1.8*(3.05-2.2)+2*1.8*(3.05-2.2)+2*2.4*(3.05-2.2)+1*5.05*(3.05-2.2)+2*4.2*(3.05-2.157)+1*3.6*(3.05-1.9)+1*1.8*(3.05-1.5)+1*1.8*(3.05-1.9)+1*3.5*(3.05-1.5)+3*3.6*(3.05-2.2)+2*2.4*(3.05-1.9)+2*2.1*(3.05-0.9)+4*0.9*(3.05-0.6)+1*0.75*(3.05-0.6))*0.858+98.4*2.45+(3*1*(3.05-2.2))*0.729+144.5*2.45+(3*1*(3.05-2.2))*0.896+127.5*2.45+(3*1*(3.05-2.2))*0.801+500.0*3.05+(10*1*(3.05-2.2)+19*0.9*(3.05-2.2)+21*0.75*(3.05-2.2)+2*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+2*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+3*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+3*1.3*(3.05-2.2)+5*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+7*1.8*(3.05-1.3)+13*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+4*1.2*(3.05-1.9)+10*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+8*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+4*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+12*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.914+443.9*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+22*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+2*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+3*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+7*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+13*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+2*0.6*(3.05-0.6)+2*1.2*(3.05-0.6))*0.889+447.7*3.05+(7*1*(3.05-2.2)+15*0.9*(3.05-2.2)+20*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+3*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+3*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+12*0.9*(3.05-0.6)+4*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.901+465.9*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+21*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+13*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+2*0.6*(3.05-0.6)+2*1.2*(3.05-0.6))*0.903+449.8*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+20*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+3*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+12*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.900+441.2*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+21*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1.2*(3.05-2.2)+3*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+13*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+2*0.6*(3.05-0.6)+2*1.2*(3.05-0.6))*0.895+397.2*3.05+(4*1*(3.05-2.2)+8*0.9*(3.05-2.2)+17*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1.2*(3.05-2.2)+2*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+2*1.6*(3.05-2.2)+1*1.3*(3.05-2.2)+2*1.8*(3.05-2.2)+3*1.8*(3.05-1.3)+6*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+1*1.2*(3.05-1.9)+5*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+3*1.5*(3.05-1.3)+2*1.5*(3.05-1.15)+1*3*(3.05-1.6)+1*1.8*(3.05-1.9)+10*0.9*(3.05-0.6)+4*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.940+354.0*3.05+(6*1*(3.05-2.2)+11*0.9*(3.05-2.2)+16*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1.2*(3.05-2.2)+2*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+3*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+3*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+4*1.8*(3.05-1.3)+8*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+2*1.2*(3.05-1.9)+6*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+5*1.5*(3.05-1.3)+3*1.5*(3.05-1.15)+1*3*(3.05-1.6)+2*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+10*0.9*(3.05-0.6)+4*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.919+82.0*2.9+(7*0.9*(3.05-2.2)+8*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+5*0.9*(3.05-0.6)+2*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.890+6.5*1.2</f>
+        <v>14146.501749599995</v>
       </c>
       <c r="F67" s="254" t="inlineStr">
         <is>
@@ -31238,7 +31238,7 @@
       </c>
       <c r="G67" s="254" t="inlineStr">
         <is>
-          <t>Openings add-back apportioned by length (150 share 0.882)</t>
+          <t>Per-floor lengths x clear heights + walling above/below openings allocated to each floor</t>
         </is>
       </c>
     </row>
@@ -31255,17 +31255,17 @@
       </c>
       <c r="C68" s="254" t="inlineStr">
         <is>
-          <t>200mm sandcrete blockwork</t>
+          <t>200mm sandcrete blockwork (floor-by-floor)</t>
         </is>
       </c>
       <c r="D68" s="254" t="inlineStr">
         <is>
-          <t>'=E65+E66*0.118</t>
+          <t>'=33.8*3.6+(1*1.8*(3.05-2.4)+6*0.9*(3.05-2.2)+1*0.9*(3.05-2.35)+1*3.2*(3.05-2.2)+6*0.75*(3.05-2.2)+2*0.7*(3.05-2.2)+3*1*(3.05-2.2)+2*0.9*(3.05-2.2)+3*1.8*(3.05-2.2)+2*1.8*(3.05-2.2)+2*2.4*(3.05-2.2)+1*5.05*(3.05-2.2)+2*4.2*(3.05-2.157)+1*3.6*(3.05-1.9)+1*1.8*(3.05-1.5)+1*1.8*(3.05-1.9)+1*3.5*(3.05-1.5)+3*3.6*(3.05-2.2)+2*2.4*(3.05-1.9)+2*2.1*(3.05-0.9)+4*0.9*(3.05-0.6)+1*0.75*(3.05-0.6))*0.142+36.6*2.45+(3*1*(3.05-2.2))*0.271+16.7*2.45+(3*1*(3.05-2.2))*0.104+31.6*2.45+(3*1*(3.05-2.2))*0.199+47.2*3.05+(10*1*(3.05-2.2)+19*0.9*(3.05-2.2)+21*0.75*(3.05-2.2)+2*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+2*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+3*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+3*1.3*(3.05-2.2)+5*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+7*1.8*(3.05-1.3)+13*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+4*1.2*(3.05-1.9)+10*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+8*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+4*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+12*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.086+55.3*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+22*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+2*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+3*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+7*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+13*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+2*0.6*(3.05-0.6)+2*1.2*(3.05-0.6))*0.111+49.2*3.05+(7*1*(3.05-2.2)+15*0.9*(3.05-2.2)+20*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+3*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+3*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+12*0.9*(3.05-0.6)+4*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.099+50.0*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+21*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+13*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+2*0.6*(3.05-0.6)+2*1.2*(3.05-0.6))*0.097+50.1*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+20*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+3*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+12*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.100+51.7*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+21*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1.2*(3.05-2.2)+3*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+13*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+2*0.6*(3.05-0.6)+2*1.2*(3.05-0.6))*0.105+25.6*3.05+(4*1*(3.05-2.2)+8*0.9*(3.05-2.2)+17*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1.2*(3.05-2.2)+2*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+2*1.6*(3.05-2.2)+1*1.3*(3.05-2.2)+2*1.8*(3.05-2.2)+3*1.8*(3.05-1.3)+6*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+1*1.2*(3.05-1.9)+5*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+3*1.5*(3.05-1.3)+2*1.5*(3.05-1.15)+1*3*(3.05-1.6)+1*1.8*(3.05-1.9)+10*0.9*(3.05-0.6)+4*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.060+31.1*3.05+(6*1*(3.05-2.2)+11*0.9*(3.05-2.2)+16*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1.2*(3.05-2.2)+2*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+3*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+3*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+4*1.8*(3.05-1.3)+8*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+2*1.2*(3.05-1.9)+6*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+5*1.5*(3.05-1.3)+3*1.5*(3.05-1.15)+1*3*(3.05-1.6)+2*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+10*0.9*(3.05-0.6)+4*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.081+10.2*2.9+(7*0.9*(3.05-2.2)+8*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+5*0.9*(3.05-0.6)+2*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.110+65.7*1.2</t>
         </is>
       </c>
       <c r="E68" s="255">
-        <f>E65+E66*0.118</f>
-        <v>1744.1390815999998</v>
+        <f>33.8*3.6+(1*1.8*(3.05-2.4)+6*0.9*(3.05-2.2)+1*0.9*(3.05-2.35)+1*3.2*(3.05-2.2)+6*0.75*(3.05-2.2)+2*0.7*(3.05-2.2)+3*1*(3.05-2.2)+2*0.9*(3.05-2.2)+3*1.8*(3.05-2.2)+2*1.8*(3.05-2.2)+2*2.4*(3.05-2.2)+1*5.05*(3.05-2.2)+2*4.2*(3.05-2.157)+1*3.6*(3.05-1.9)+1*1.8*(3.05-1.5)+1*1.8*(3.05-1.9)+1*3.5*(3.05-1.5)+3*3.6*(3.05-2.2)+2*2.4*(3.05-1.9)+2*2.1*(3.05-0.9)+4*0.9*(3.05-0.6)+1*0.75*(3.05-0.6))*0.142+36.6*2.45+(3*1*(3.05-2.2))*0.271+16.7*2.45+(3*1*(3.05-2.2))*0.104+31.6*2.45+(3*1*(3.05-2.2))*0.199+47.2*3.05+(10*1*(3.05-2.2)+19*0.9*(3.05-2.2)+21*0.75*(3.05-2.2)+2*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+2*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+3*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+3*1.3*(3.05-2.2)+5*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+7*1.8*(3.05-1.3)+13*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+4*1.2*(3.05-1.9)+10*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+8*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+4*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+12*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.086+55.3*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+22*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+2*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+3*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+7*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+13*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+2*0.6*(3.05-0.6)+2*1.2*(3.05-0.6))*0.111+49.2*3.05+(7*1*(3.05-2.2)+15*0.9*(3.05-2.2)+20*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+3*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+3*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+12*0.9*(3.05-0.6)+4*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.099+50.0*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+21*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+3*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+5*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+13*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+2*0.6*(3.05-0.6)+2*1.2*(3.05-0.6))*0.097+50.1*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+20*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+3*1.2*(3.05-2.2)+3*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+3*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+12*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.100+51.7*3.05+(8*1*(3.05-2.2)+15*0.9*(3.05-2.2)+21*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1.2*(3.05-2.2)+3*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+4*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+4*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+6*1.8*(3.05-1.3)+10*0.9*(3.05-1.3)+2*1.8*(3.05-1.6)+3*1.2*(3.05-1.9)+8*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+6*1.5*(3.05-1.3)+4*1.5*(3.05-1.15)+1*2.4*(3.05-1.3)+1*3*(3.05-1.6)+3*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+1*1.45*(3.05-1.9)+13*0.9*(3.05-0.6)+5*0.75*(3.05-0.6)+2*0.6*(3.05-0.6)+2*1.2*(3.05-0.6))*0.105+25.6*3.05+(4*1*(3.05-2.2)+8*0.9*(3.05-2.2)+17*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1.2*(3.05-2.2)+2*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+2*1.6*(3.05-2.2)+1*1.3*(3.05-2.2)+2*1.8*(3.05-2.2)+3*1.8*(3.05-1.3)+6*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+1*1.2*(3.05-1.9)+5*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+3*1.5*(3.05-1.3)+2*1.5*(3.05-1.15)+1*3*(3.05-1.6)+1*1.8*(3.05-1.9)+10*0.9*(3.05-0.6)+4*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.060+31.1*3.05+(6*1*(3.05-2.2)+11*0.9*(3.05-2.2)+16*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1.2*(3.05-2.2)+2*1*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+1*1.5*(3.05-2.2)+2*0.9*(3.05-2.2)+4*0.75*(3.05-2.2)+1*0.45*(3.05-2.2)+3*0.6*(3.05-2.2)+1*3*(3.05-2.2)+3*1.6*(3.05-2.2)+2*1.3*(3.05-2.2)+3*1.8*(3.05-2.2)+1*1.2*(3.05-2.2)+4*1.8*(3.05-1.3)+8*0.9*(3.05-1.3)+1*1.8*(3.05-1.6)+2*1.2*(3.05-1.9)+6*1.2*(3.05-1.15)+1*1.2*(3.05-1.2)+5*1.5*(3.05-1.3)+3*1.5*(3.05-1.15)+1*3*(3.05-1.6)+2*1.8*(3.05-1.9)+1*0.75*(3.05-1.3)+10*0.9*(3.05-0.6)+4*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.081+10.2*2.9+(7*0.9*(3.05-2.2)+8*0.75*(3.05-2.2)+1*0.7*(3.05-2.2)+2*1*(3.05-2.2)+1*0.9*(3.05-2.2)+5*0.9*(3.05-0.6)+2*0.75*(3.05-0.6)+1*0.6*(3.05-0.6)+1*1.2*(3.05-0.6))*0.110+65.7*1.2</f>
+        <v>1708.1694503999997</v>
       </c>
       <c r="F68" s="254" t="inlineStr">
         <is>
@@ -31578,17 +31578,17 @@
       </c>
       <c r="C78" s="254" t="inlineStr">
         <is>
-          <t>50x50 matte R11 porcelain - staircases (treads, risers, landings): 22 storey-flights x 31.74 m2</t>
+          <t>50x50 matte R11 porcelain - staircases (treads, risers, landings): 23 storey-flights (main 11, emergency 12) x 31.74 m2</t>
         </is>
       </c>
       <c r="D78" s="254" t="inlineStr">
         <is>
-          <t>'=(2*1.8*3.0+22*0.15*1.8+2.2*3.75+1.8*3.75)*22</t>
+          <t>'=(2*1.8*3.0+22*0.15*1.8+2.2*3.75+1.8*3.75)*23</t>
         </is>
       </c>
       <c r="E78" s="255">
-        <f>(2*1.8*3.0+22*0.15*1.8+2.2*3.75+1.8*3.75)*22</f>
-        <v>698.2800000000001</v>
+        <f>(2*1.8*3.0+22*0.15*1.8+2.2*3.75+1.8*3.75)*23</f>
+        <v>730.0200000000001</v>
       </c>
       <c r="F78" s="254" t="inlineStr">
         <is>
@@ -31867,12 +31867,12 @@
       </c>
       <c r="D86" s="254" t="inlineStr">
         <is>
-          <t>'=E84+(2*1.8*3.0+22*0.15*1.8+2.2*3.75+1.8*3.75)*22</t>
+          <t>'=E84+(2*1.8*3.0+22*0.15*1.8+2.2*3.75+1.8*3.75)*23</t>
         </is>
       </c>
       <c r="E86" s="255">
-        <f>E84+(2*1.8*3.0+22*0.15*1.8+2.2*3.75+1.8*3.75)*22</f>
-        <v>8342.48</v>
+        <f>E84+(2*1.8*3.0+22*0.15*1.8+2.2*3.75+1.8*3.75)*23</f>
+        <v>8374.22</v>
       </c>
       <c r="F86" s="254" t="inlineStr">
         <is>
@@ -32316,17 +32316,17 @@
       </c>
       <c r="C101" s="254" t="inlineStr">
         <is>
-          <t>Pairs 100mm brass butt hinges: 1.5 pairs per timber leaf (299 leaves)</t>
+          <t>Pairs 100mm brass butt hinges: 1.5 pairs per timber leaf (299 leaves), rounded up per floor</t>
         </is>
       </c>
       <c r="D101" s="254" t="inlineStr">
         <is>
-          <t>'=ROUNDUP(1.5*(126+1+172),0)</t>
+          <t>'=20+60+56+53+54+53+54+38+41+23</t>
         </is>
       </c>
       <c r="E101" s="255">
-        <f>ROUNDUP(1.5*(126+1+172),0)</f>
-        <v>449.0</v>
+        <f>20+60+56+53+54+53+54+38+41+23</f>
+        <v>452.0</v>
       </c>
       <c r="F101" s="254" t="inlineStr">
         <is>

</xml_diff>